<commit_message>
Refresh workbook: correct Caribbean Cement split to the live-engine figures
The prior export still had the stale standalone-model numbers (105.9/103.0/97.9,
declining) that Section 1 of the Driver Report has since been corrected away
from (106.7/104.5/109.5, rising into FY2028 -- see commit 09ea795). Recalculated,
zero formula errors.
</commit_message>
<xml_diff>
--- a/JPS_Driver_Report_Data_FY2026-28.xlsx
+++ b/JPS_Driver_Report_Data_FY2026-28.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">JPS Sales Forecast — Rate Class Totals (GWh)</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: Driver Forecast engine, live-verified 2026-09-08. FY2025-26 actual/closed, FY2027-28 forecast.</t>
+    <t xml:space="preserve">Source: Driver Forecast engine, live-verified 2026-09-10. FY2025-26 actual/closed, FY2027-28 forecast. Caribbean Cement is this account's own live chain (Section 1 note); a separate standalone model used elsewhere does not tie to it.</t>
   </si>
   <si>
     <t xml:space="preserve">Rate Class</t>
@@ -1344,21 +1344,21 @@
         <v>16</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>105.9</v>
+        <v>106.7</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>103</v>
+        <v>104.5</v>
       </c>
       <c r="D15" s="7" t="n">
         <f aca="false">(C15-B15)/B15</f>
-        <v>-0.0273843248347498</v>
+        <v>-0.020618556701031</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>97.9</v>
+        <v>109.5</v>
       </c>
       <c r="F15" s="7" t="n">
         <f aca="false">(E15-C15)/C15</f>
-        <v>-0.0495145631067961</v>
+        <v>0.0478468899521531</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1366,21 +1366,21 @@
         <v>17</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>239.7</v>
+        <v>239.1</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>297.8</v>
+        <v>296.8</v>
       </c>
       <c r="D16" s="7" t="n">
         <f aca="false">(C16-B16)/B16</f>
-        <v>0.242386316228619</v>
+        <v>0.241321622751987</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>335.6</v>
+        <v>324.4</v>
       </c>
       <c r="F16" s="7" t="n">
         <f aca="false">(E16-C16)/C16</f>
-        <v>0.126930826057757</v>
+        <v>0.0929919137466306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>